<commit_message>
Update collectors: aggregates S3 cleanup, cambridge GUI/processor enhancements, rich text utils
</commit_message>
<xml_diff>
--- a/aggregates/input/Aggregates Price List v2.xlsx
+++ b/aggregates/input/Aggregates Price List v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/moosemarketer/Code/garoppos/collectors/aggregates/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{259C1841-8194-5048-A6E5-B587217BFD97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BC92EDC-11CC-D54D-A6B3-4B9FCDB65664}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="35440" windowHeight="19800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="97">
   <si>
     <t>Yard</t>
   </si>
@@ -242,9 +242,6 @@
   </si>
   <si>
     <t>Jersey Yellow</t>
-  </si>
-  <si>
-    <t>Light Grey</t>
   </si>
   <si>
     <t>Concrete</t>
@@ -964,7 +961,7 @@
         <v>53</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>15</v>
@@ -999,10 +996,10 @@
         <v>5071</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E2" s="8">
         <v>33</v>
@@ -1011,7 +1008,7 @@
         <v>19</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="I2" s="1" t="s">
         <v>0</v>
@@ -1020,7 +1017,7 @@
         <v>1</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="19">
@@ -1031,10 +1028,10 @@
         <v>5071</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E3" s="8">
         <v>33</v>
@@ -1043,7 +1040,7 @@
         <v>19</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="I3" s="1" t="s">
         <v>0</v>
@@ -1063,10 +1060,10 @@
         <v>5071</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E4" s="8">
         <v>33</v>
@@ -1075,7 +1072,7 @@
         <v>19</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="I4" s="1" t="s">
         <v>0</v>
@@ -1084,7 +1081,7 @@
         <v>1</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="19">
@@ -1095,10 +1092,10 @@
         <v>5071</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E5" s="8">
         <v>19.5</v>
@@ -1116,7 +1113,7 @@
         <v>1</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="19">
@@ -1127,10 +1124,10 @@
         <v>5071</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E6" s="8">
         <v>38</v>
@@ -1159,10 +1156,10 @@
         <v>5071</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E7" s="8">
         <v>23.5</v>
@@ -1191,10 +1188,10 @@
         <v>5071</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E8" s="8">
         <v>28.5</v>
@@ -1220,7 +1217,7 @@
         <v>18163</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>2</v>
@@ -1246,7 +1243,7 @@
         <v>24605</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>4</v>
@@ -1272,7 +1269,7 @@
         <v>13878</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D11" s="1" t="s">
         <v>6</v>
@@ -1298,7 +1295,7 @@
         <v>24603</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D12" s="1" t="s">
         <v>7</v>
@@ -1324,7 +1321,7 @@
         <v>24604</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D13" s="1" t="s">
         <v>8</v>
@@ -1353,10 +1350,10 @@
         <v>24601</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E14" s="8">
         <v>24</v>
@@ -1365,7 +1362,7 @@
         <v>12.5</v>
       </c>
       <c r="G14" s="6" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I14" s="1" t="s">
         <v>5</v>
@@ -1385,10 +1382,10 @@
         <v>24601</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E15" s="8">
         <v>23</v>
@@ -1397,7 +1394,7 @@
         <v>10.5</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="I15" s="1" t="s">
         <v>5</v>
@@ -1417,10 +1414,10 @@
         <v>24601</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E16" s="8">
         <v>35</v>
@@ -1429,7 +1426,7 @@
         <v>21</v>
       </c>
       <c r="G16" s="6" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="I16" s="1" t="s">
         <v>5</v>
@@ -1446,7 +1443,7 @@
         <v>24608</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D17" s="1" t="s">
         <v>52</v>
@@ -1464,7 +1461,7 @@
         <v>3</v>
       </c>
       <c r="K17" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="18" spans="1:11" ht="19">
@@ -1475,10 +1472,10 @@
         <v>24612</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E18" s="8">
         <v>45</v>
@@ -1499,7 +1496,7 @@
         <v>3</v>
       </c>
       <c r="K18" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="19" spans="1:11" ht="19">
@@ -1510,10 +1507,10 @@
         <v>24612</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E19" s="8">
         <v>57</v>
@@ -1545,10 +1542,10 @@
         <v>24613</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E20" s="8">
         <v>54</v>
@@ -1577,10 +1574,10 @@
         <v>24613</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E21" s="8">
         <v>54</v>
@@ -1609,10 +1606,10 @@
         <v>24614</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E22" s="8">
         <v>93</v>
@@ -1641,10 +1638,10 @@
         <v>24614</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E23" s="8">
         <v>93</v>
@@ -1673,10 +1670,10 @@
         <v>24614</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E24" s="8">
         <v>95</v>
@@ -1705,10 +1702,10 @@
         <v>24614</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E25" s="8">
         <v>95</v>
@@ -1737,10 +1734,10 @@
         <v>24614</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E26" s="8">
         <v>95</v>
@@ -1758,7 +1755,7 @@
         <v>14</v>
       </c>
       <c r="K26" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="27" spans="1:11" ht="19">
@@ -1769,10 +1766,10 @@
         <v>24616</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E27" s="8">
         <v>46</v>
@@ -1801,19 +1798,16 @@
         <v>24616</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E28" s="8">
         <v>45</v>
       </c>
       <c r="F28" s="8">
         <v>31.5</v>
-      </c>
-      <c r="G28" s="6" t="s">
-        <v>68</v>
       </c>
       <c r="H28" s="8" t="s">
         <v>57</v>
@@ -1833,10 +1827,10 @@
         <v>24617</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E29" s="8">
         <v>46</v>
@@ -1851,7 +1845,7 @@
         <v>5</v>
       </c>
       <c r="K29" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="30" spans="1:11" ht="19">
@@ -1862,10 +1856,10 @@
         <v>24615</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E30" s="8">
         <v>49</v>
@@ -1883,7 +1877,7 @@
         <v>3</v>
       </c>
       <c r="K30" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="31" spans="1:11" ht="19">
@@ -1894,10 +1888,10 @@
         <v>24615</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E31" s="8">
         <v>49</v>
@@ -1923,10 +1917,10 @@
         <v>24622</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D32" s="6" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E32" s="8">
         <v>40</v>
@@ -1952,10 +1946,10 @@
         <v>24623</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E33" s="8">
         <v>40</v>
@@ -1981,10 +1975,10 @@
         <v>24611</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D34" s="6" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E34" s="8">
         <v>98</v>
@@ -2013,10 +2007,10 @@
         <v>24611</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E35" s="8">
         <v>98</v>
@@ -2045,10 +2039,10 @@
         <v>24611</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D36" s="6" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E36" s="8">
         <v>98</v>
@@ -2074,10 +2068,10 @@
         <v>29273</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E37" s="8">
         <v>84</v>
@@ -2103,10 +2097,10 @@
         <v>24705</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E38" s="8">
         <v>51</v>
@@ -2132,7 +2126,7 @@
         <v>30120</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D39" s="1" t="s">
         <v>12</v>

</xml_diff>